<commit_message>
store/map.edf bells 8 banner + fix remove buffer on banner
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/neutralB.xlsx
+++ b/gu_in/Map.edf/neutralB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1227532B-CEAE-46B4-A843-0761483BCB2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224A919F-6DDA-4B11-8DF0-6A5160F0F596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12720" yWindow="1020" windowWidth="10110" windowHeight="11205" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -22,12 +22,23 @@
     <sheet name="Other Dummy" sheetId="7" r:id="rId7"/>
     <sheet name="Zones" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2267" uniqueCount="1107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2283" uniqueCount="1123">
   <si>
     <t>char[32]</t>
   </si>
@@ -3348,6 +3359,54 @@
   </si>
   <si>
     <t>bd131B3</t>
+  </si>
+  <si>
+    <t>sd131C5</t>
+  </si>
+  <si>
+    <t>bd131C5</t>
+  </si>
+  <si>
+    <t>sd131C6</t>
+  </si>
+  <si>
+    <t>bd131C6</t>
+  </si>
+  <si>
+    <t>sd131C7</t>
+  </si>
+  <si>
+    <t>bd131C7</t>
+  </si>
+  <si>
+    <t>sd131C8</t>
+  </si>
+  <si>
+    <t>bd131C8</t>
+  </si>
+  <si>
+    <t>sd131C9</t>
+  </si>
+  <si>
+    <t>bd131C9</t>
+  </si>
+  <si>
+    <t>sd131D0</t>
+  </si>
+  <si>
+    <t>bd131D0</t>
+  </si>
+  <si>
+    <t>sd131D1</t>
+  </si>
+  <si>
+    <t>bd131D1</t>
+  </si>
+  <si>
+    <t>sd131D2</t>
+  </si>
+  <si>
+    <t>bd131D2</t>
   </si>
 </sst>
 </file>
@@ -32552,7 +32611,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H211"/>
+  <dimension ref="A1:H227"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -38038,6 +38097,422 @@
         <v>20</v>
       </c>
       <c r="H211" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="212" spans="1:8">
+      <c r="A212" s="1" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B212" s="1">
+        <v>140</v>
+      </c>
+      <c r="C212" s="1">
+        <v>-6064</v>
+      </c>
+      <c r="D212" s="1">
+        <v>550</v>
+      </c>
+      <c r="E212" s="1">
+        <v>6107</v>
+      </c>
+      <c r="F212" s="1">
+        <v>20</v>
+      </c>
+      <c r="G212" s="1">
+        <v>20</v>
+      </c>
+      <c r="H212" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="213" spans="1:8">
+      <c r="A213" s="1" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B213" s="1">
+        <v>140</v>
+      </c>
+      <c r="C213" s="1">
+        <v>-6064</v>
+      </c>
+      <c r="D213" s="1">
+        <v>550</v>
+      </c>
+      <c r="E213" s="1">
+        <v>6107</v>
+      </c>
+      <c r="F213" s="1">
+        <v>20</v>
+      </c>
+      <c r="G213" s="1">
+        <v>20</v>
+      </c>
+      <c r="H213" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="214" spans="1:8">
+      <c r="A214" s="1" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B214" s="1">
+        <v>140</v>
+      </c>
+      <c r="C214" s="1">
+        <v>-6181</v>
+      </c>
+      <c r="D214" s="1">
+        <v>550</v>
+      </c>
+      <c r="E214" s="1">
+        <v>6050</v>
+      </c>
+      <c r="F214" s="1">
+        <v>20</v>
+      </c>
+      <c r="G214" s="1">
+        <v>20</v>
+      </c>
+      <c r="H214" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="215" spans="1:8">
+      <c r="A215" s="1" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B215" s="1">
+        <v>140</v>
+      </c>
+      <c r="C215" s="1">
+        <v>-6181</v>
+      </c>
+      <c r="D215" s="1">
+        <v>550</v>
+      </c>
+      <c r="E215" s="1">
+        <v>6050</v>
+      </c>
+      <c r="F215" s="1">
+        <v>20</v>
+      </c>
+      <c r="G215" s="1">
+        <v>20</v>
+      </c>
+      <c r="H215" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8">
+      <c r="A216" s="1" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B216" s="1">
+        <v>140</v>
+      </c>
+      <c r="C216" s="1">
+        <v>-6100</v>
+      </c>
+      <c r="D216" s="1">
+        <v>550</v>
+      </c>
+      <c r="E216" s="1">
+        <v>5993</v>
+      </c>
+      <c r="F216" s="1">
+        <v>20</v>
+      </c>
+      <c r="G216" s="1">
+        <v>20</v>
+      </c>
+      <c r="H216" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="217" spans="1:8">
+      <c r="A217" s="1" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B217" s="1">
+        <v>140</v>
+      </c>
+      <c r="C217" s="1">
+        <v>-6100</v>
+      </c>
+      <c r="D217" s="1">
+        <v>550</v>
+      </c>
+      <c r="E217" s="1">
+        <v>5993</v>
+      </c>
+      <c r="F217" s="1">
+        <v>20</v>
+      </c>
+      <c r="G217" s="1">
+        <v>20</v>
+      </c>
+      <c r="H217" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="218" spans="1:8">
+      <c r="A218" s="1" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B218" s="1">
+        <v>140</v>
+      </c>
+      <c r="C218" s="1">
+        <v>-6018</v>
+      </c>
+      <c r="D218" s="1">
+        <v>550</v>
+      </c>
+      <c r="E218" s="1">
+        <v>5934</v>
+      </c>
+      <c r="F218" s="1">
+        <v>20</v>
+      </c>
+      <c r="G218" s="1">
+        <v>20</v>
+      </c>
+      <c r="H218" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="219" spans="1:8">
+      <c r="A219" s="1" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B219" s="1">
+        <v>140</v>
+      </c>
+      <c r="C219" s="1">
+        <v>-6018</v>
+      </c>
+      <c r="D219" s="1">
+        <v>550</v>
+      </c>
+      <c r="E219" s="1">
+        <v>5934</v>
+      </c>
+      <c r="F219" s="1">
+        <v>20</v>
+      </c>
+      <c r="G219" s="1">
+        <v>20</v>
+      </c>
+      <c r="H219" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="220" spans="1:8">
+      <c r="A220" s="1" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B220" s="1">
+        <v>140</v>
+      </c>
+      <c r="C220" s="1">
+        <v>-6393</v>
+      </c>
+      <c r="D220" s="1">
+        <v>550</v>
+      </c>
+      <c r="E220" s="1">
+        <v>5923</v>
+      </c>
+      <c r="F220" s="1">
+        <v>20</v>
+      </c>
+      <c r="G220" s="1">
+        <v>20</v>
+      </c>
+      <c r="H220" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8">
+      <c r="A221" s="1" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B221" s="1">
+        <v>140</v>
+      </c>
+      <c r="C221" s="1">
+        <v>-6393</v>
+      </c>
+      <c r="D221" s="1">
+        <v>550</v>
+      </c>
+      <c r="E221" s="1">
+        <v>5923</v>
+      </c>
+      <c r="F221" s="1">
+        <v>20</v>
+      </c>
+      <c r="G221" s="1">
+        <v>20</v>
+      </c>
+      <c r="H221" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8">
+      <c r="A222" s="1" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B222" s="1">
+        <v>140</v>
+      </c>
+      <c r="C222" s="1">
+        <v>-6311</v>
+      </c>
+      <c r="D222" s="1">
+        <v>550</v>
+      </c>
+      <c r="E222" s="1">
+        <v>5865</v>
+      </c>
+      <c r="F222" s="1">
+        <v>20</v>
+      </c>
+      <c r="G222" s="1">
+        <v>20</v>
+      </c>
+      <c r="H222" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8">
+      <c r="A223" s="1" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B223" s="1">
+        <v>140</v>
+      </c>
+      <c r="C223" s="1">
+        <v>-6311</v>
+      </c>
+      <c r="D223" s="1">
+        <v>550</v>
+      </c>
+      <c r="E223" s="1">
+        <v>5865</v>
+      </c>
+      <c r="F223" s="1">
+        <v>20</v>
+      </c>
+      <c r="G223" s="1">
+        <v>20</v>
+      </c>
+      <c r="H223" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8">
+      <c r="A224" s="1" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B224" s="1">
+        <v>140</v>
+      </c>
+      <c r="C224" s="1">
+        <v>-6229</v>
+      </c>
+      <c r="D224" s="1">
+        <v>550</v>
+      </c>
+      <c r="E224" s="1">
+        <v>5807</v>
+      </c>
+      <c r="F224" s="1">
+        <v>20</v>
+      </c>
+      <c r="G224" s="1">
+        <v>20</v>
+      </c>
+      <c r="H224" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8">
+      <c r="A225" s="1" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B225" s="1">
+        <v>140</v>
+      </c>
+      <c r="C225" s="1">
+        <v>-6229</v>
+      </c>
+      <c r="D225" s="1">
+        <v>550</v>
+      </c>
+      <c r="E225" s="1">
+        <v>5807</v>
+      </c>
+      <c r="F225" s="1">
+        <v>20</v>
+      </c>
+      <c r="G225" s="1">
+        <v>20</v>
+      </c>
+      <c r="H225" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="226" spans="1:8">
+      <c r="A226" s="1" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B226" s="1">
+        <v>140</v>
+      </c>
+      <c r="C226" s="1">
+        <v>-6147</v>
+      </c>
+      <c r="D226" s="1">
+        <v>550</v>
+      </c>
+      <c r="E226" s="1">
+        <v>5751</v>
+      </c>
+      <c r="F226" s="1">
+        <v>20</v>
+      </c>
+      <c r="G226" s="1">
+        <v>20</v>
+      </c>
+      <c r="H226" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8">
+      <c r="A227" s="1" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B227" s="1">
+        <v>140</v>
+      </c>
+      <c r="C227" s="1">
+        <v>-6147</v>
+      </c>
+      <c r="D227" s="1">
+        <v>550</v>
+      </c>
+      <c r="E227" s="1">
+        <v>5751</v>
+      </c>
+      <c r="F227" s="1">
+        <v>20</v>
+      </c>
+      <c r="G227" s="1">
+        <v>20</v>
+      </c>
+      <c r="H227" s="1">
         <v>20</v>
       </c>
     </row>

</xml_diff>